<commit_message>
CORE-000019 edit: added output variables
</commit_message>
<xml_diff>
--- a/rules/CORE-000019/negative/01/data/unit-test-coreid-CG0311-negative.xlsx
+++ b/rules/CORE-000019/negative/01/data/unit-test-coreid-CG0311-negative.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\CORE-000019\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A678BA0D-27FD-48A5-9B3D-0E3051BA30BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{195A042F-5E7A-4FB6-9BB1-492A13071BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="89">
   <si>
     <t>Product</t>
   </si>
@@ -304,6 +304,9 @@
   </si>
   <si>
     <t>variable_label</t>
+  </si>
+  <si>
+    <t>variable_name</t>
   </si>
 </sst>
 </file>
@@ -392,7 +395,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -426,6 +429,10 @@
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -816,8 +823,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -839,7 +849,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -852,16 +862,16 @@
       <c r="D2">
         <v>3</v>
       </c>
-      <c r="E2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F2" s="10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="120" x14ac:dyDescent="0.25">
+      <c r="E2" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
@@ -870,92 +880,212 @@
         <v>18</v>
       </c>
       <c r="D3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E3" t="s">
         <v>87</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
       </c>
       <c r="D4">
-        <v>3</v>
-      </c>
-      <c r="E4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
       </c>
       <c r="D5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E5" t="s">
         <v>87</v>
       </c>
-      <c r="F5" s="13" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+      <c r="F5" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C6" t="s">
         <v>18</v>
       </c>
       <c r="D6">
-        <v>5</v>
-      </c>
-      <c r="E6" t="s">
-        <v>87</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>62</v>
+        <v>3</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>85</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
         <v>18</v>
       </c>
       <c r="D7">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E7" t="s">
         <v>87</v>
       </c>
       <c r="F7" s="10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8">
+        <v>6</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9">
+        <v>6</v>
+      </c>
+      <c r="E9" t="s">
+        <v>87</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>5</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10">
+        <v>5</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>5</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11" t="s">
+        <v>87</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>6</v>
+      </c>
+      <c r="B12" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12">
+        <v>5</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>6</v>
+      </c>
+      <c r="B13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13">
+        <v>5</v>
+      </c>
+      <c r="E13" t="s">
+        <v>87</v>
+      </c>
+      <c r="F13" s="10" t="s">
         <v>84</v>
       </c>
     </row>

</xml_diff>